<commit_message>
Mark eight outreach emails as sent on 20 September 2026
All eight approved applications went out with the CV attached. Tracker rows
now carry Email Sent, Date Sent, CV Attached, status Sent, and a follow-up
date of 28 September, six working days out per the tracker's own guidance
that most replies come from the second email.

Recipients: Gudz, MoreTasks, C11 Aura, Meesho, Elda, The Bijou Box, Ugaoo
and iCARRY. The five cold contacts emailed in May 2026 for the same role
remain untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NtzogBerrfgjBtAVFPBbXL
</commit_message>
<xml_diff>
--- a/outreach/Outreach_Tracker.xlsx
+++ b/outreach/Outreach_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outreach" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do Not Contact" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Outreach" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Do Not Contact" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="How to use" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -669,7 +669,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>MoreTasks</t>
@@ -728,14 +732,26 @@
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr"/>
-      <c r="S2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -749,7 +765,7 @@
       <c r="V2" s="2" t="inlineStr"/>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X2" s="3" t="inlineStr">
@@ -759,7 +775,11 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>C11 Aura</t>
@@ -814,14 +834,26 @@
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -835,7 +867,7 @@
       <c r="V3" s="2" t="inlineStr"/>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X3" s="3" t="inlineStr">
@@ -845,7 +877,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
           <t>The Bijou Box</t>
@@ -904,14 +940,26 @@
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr"/>
-      <c r="P4" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -925,7 +973,7 @@
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X4" s="3" t="inlineStr">
@@ -935,7 +983,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Gudz</t>
@@ -994,14 +1046,26 @@
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr"/>
-      <c r="P5" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1015,7 +1079,7 @@
       <c r="V5" s="2" t="inlineStr"/>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X5" s="3" t="inlineStr">
@@ -1025,7 +1089,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Meesho</t>
@@ -1084,14 +1152,26 @@
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr"/>
-      <c r="P6" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="inlineStr"/>
-      <c r="S6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1105,7 +1185,7 @@
       <c r="V6" s="2" t="inlineStr"/>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X6" s="3" t="inlineStr">
@@ -1115,7 +1195,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Elda</t>
@@ -1170,14 +1254,26 @@
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr"/>
-      <c r="P7" s="2" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="Q7" s="2" t="inlineStr"/>
       <c r="R7" s="2" t="inlineStr"/>
-      <c r="S7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1191,7 +1287,7 @@
       <c r="V7" s="2" t="inlineStr"/>
       <c r="W7" s="2" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X7" s="3" t="inlineStr">
@@ -1373,7 +1469,11 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Ugaoo</t>
@@ -1432,14 +1532,26 @@
       <c r="M10" s="4" t="inlineStr"/>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O10" s="4" t="inlineStr"/>
-      <c r="P10" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="Q10" s="4" t="inlineStr"/>
       <c r="R10" s="4" t="inlineStr"/>
-      <c r="S10" s="4" t="inlineStr"/>
+      <c r="S10" s="4" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
       <c r="T10" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1453,7 +1565,7 @@
       <c r="V10" s="4" t="inlineStr"/>
       <c r="W10" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X10" s="5" t="inlineStr">
@@ -1721,7 +1833,11 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
           <t>iCARRY</t>
@@ -1776,14 +1892,26 @@
       <c r="M14" s="4" t="inlineStr"/>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="O14" s="4" t="inlineStr"/>
-      <c r="P14" s="4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="Q14" s="4" t="inlineStr"/>
       <c r="R14" s="4" t="inlineStr"/>
-      <c r="S14" s="4" t="inlineStr"/>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
       <c r="T14" s="4" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -1797,7 +1925,7 @@
       <c r="V14" s="4" t="inlineStr"/>
       <c r="W14" s="4" t="inlineStr">
         <is>
-          <t>Ready to Send</t>
+          <t>Sent</t>
         </is>
       </c>
       <c r="X14" s="5" t="inlineStr">

</xml_diff>